<commit_message>
500 collage  limit set
</commit_message>
<xml_diff>
--- a/exports/colleges/10343_christian-medical-college-cmc-vellore.xlsx
+++ b/exports/colleges/10343_christian-medical-college-cmc-vellore.xlsx
@@ -605,19 +605,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="39" customWidth="1" min="3" max="3"/>
-    <col width="39" customWidth="1" min="4" max="4"/>
-    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
   </cols>
@@ -707,12 +707,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.6 Lakhs</t>
+          <t>1.6 L</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>10+2 with 45%</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>BPT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -769,12 +769,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.36 Lakhs</t>
+          <t>1.36 L</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>10+2 with 35%</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4 Lakhs</t>
+          <t>1.4 L</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4 Years</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>10+2 with 35%</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2.5 Lakhs</t>
+          <t>2.5 L</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3 Years</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -908,17 +908,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>MBBS + NEET PG</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Tamil Nadu NEET PG Counselling, NEET PG</t>
+          <t>NEET PG</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>18 Mar - 21 Mar 2026</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MBBS</t>
+          <t>M.B.B.S.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -950,17 +950,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>M.B.B.S.</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2.9 Lakhs</t>
+          <t>2.9 L</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>5 Years</t>
+          <t>5 years</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -970,17 +970,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>10+2 with 50% + NEET-UG</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NEET, Tamil Nadu NEET Counselling</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1002,27 +1002,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B.Sc</t>
+          <t>M.Ch</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B.Sc. Nursing</t>
+          <t>Master of Chirurgiae [M.Ch]</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>B.Sc. Nursing</t>
+          <t>Master of Chirurgiae [M.Ch]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.6 Lakhs</t>
+          <t>2.76 L - 3.07 L</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3 Years</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1032,17 +1032,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>10+2 with 45%</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>NEET SS</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>10 Mar - 03 Apr 2026</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -1064,27 +1064,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BPT</t>
+          <t>M.Sc</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BPT</t>
+          <t>Master of Science [M.Sc]</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BPT</t>
+          <t>Master of Science [M.Sc]</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.36 Lakhs</t>
+          <t>68,185 - 1.03 L</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1094,17 +1094,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>10+2 with 50%</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>IIT JAM</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>30 Sept - 01 Oct 2026</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1126,27 +1126,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B.Sc</t>
+          <t>Post Doctoral Fellowship Programme</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B.Sc.</t>
+          <t>Post Doctoral Fellowship Programme</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B.Sc.</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.35 – 1.42 lakh</t>
+          <t>62000</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3 Years</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -1188,27 +1188,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2.5 Lakh</t>
+          <t>2.76 L</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3 Years</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1218,12 +1218,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>MBBS + NEET PG</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NEET PG</t>
+          <t>NEET SS</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -1250,27 +1250,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MBBS</t>
+          <t>Bachelor of Occupational Therapy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MBBS</t>
+          <t>Bachelor of Occupational Therapy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MBBS</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2.9 Lakh</t>
+          <t>1.46 L</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5 Years 6 Months</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1280,17 +1280,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>10+2 with 50% + NEET-UG</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NEET</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1312,27 +1312,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>M.Ch</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>M.Ch</t>
+          <t>Doctorate of Medicine [DM]</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>M.Ch</t>
+          <t>Doctorate of Medicine [DM]</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.76–3.07 Lakh</t>
+          <t>2.76 L</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1342,12 +1342,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Post-Graduation + NEET SS</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>NEET SS</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -1374,27 +1374,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>Master of Surgery [MS]</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>M.Sc</t>
+          <t>Master of Surgery [MS]</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>68,185 – 1.03 Lakh</t>
+          <t>2.5 L</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2 Years</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1404,17 +1404,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>B.Sc. Nursing with 55%</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>IIT JAM</t>
+          <t>NEET PG</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>17 Apr - 07 Jul 2026</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1436,27 +1436,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Fellowship</t>
+          <t>MPH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fellowship</t>
+          <t>Master of Public Health [MPH]</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Fellowship</t>
+          <t>Master of Public Health [MPH]</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>62,000</t>
+          <t>1.41 L</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3-5 Years</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1466,12 +1466,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>MD/DNB</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>GATE / UGC NET</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Doctorate</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1498,27 +1498,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tuition Fee</t>
+          <t>BASLP</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tuition Fee</t>
+          <t>Bachelor in Audiology and Speech - Language Pathology [BASLP]</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tuition Fee</t>
+          <t>Bachelor in Audiology and Speech - Language Pathology [BASLP]</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3,000</t>
+          <t>1.4 L</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1560,27 +1560,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>One-time College Fee (at admission)</t>
+          <t>GNM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>One-time College Fee (at admission)</t>
+          <t>General Nursing and Midwifery [GNM]</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>One-time College Fee (at admission)</t>
+          <t>General Nursing and Midwifery [GNM]</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>12,260</t>
+          <t>1.12 L</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1622,27 +1622,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Other Annual Fees</t>
+          <t>Post Graduate Diploma</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Other Annual Fees</t>
+          <t>Post Graduate Diploma</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Other Annual Fees</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>54,095</t>
+          <t>20,060 - 39,117</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1684,27 +1684,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>One-time University Payment</t>
+          <t>MHA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>One-time University Payment</t>
+          <t>Master in Hospital Administration [MHA]</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>One-time University Payment</t>
+          <t>Master in Hospital Administration [MHA]</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>14,975</t>
+          <t>1.63 L</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1746,27 +1746,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1st Year Total</t>
+          <t>B.Optom</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1st Year Total</t>
+          <t>Bachelor of Optometry [B.Optom]</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1st Year Total</t>
+          <t>Bachelor of Optometry [B.Optom]</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>84,330</t>
+          <t>1.4 L</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1808,32 +1808,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Admission year Chrages</t>
+          <t>Post Graduate Diploma</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Admission year Chrages</t>
+          <t>Post Graduate Diploma</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Admission year Chrages</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>26,410</t>
+          <t>75,000 - 1 L</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Full Time</t>
+          <t>Part Time</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1870,27 +1870,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Charges for Other Years</t>
+          <t>Diploma</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Charges for Other Years</t>
+          <t>Diploma</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Charges for Other Years</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>17,310</t>
+          <t>20,131 - 3.15 L</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 Apr - 13 Jun 2026</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1932,27 +1932,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Other Fees</t>
+          <t>Post Basic Diploma</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Other Fees</t>
+          <t>Post Basic Diploma</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Other Fees</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>3500 (Electricity)</t>
+          <t>31,690</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -1994,27 +1994,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tuition Fee</t>
+          <t>B.Sc</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tuition Fee</t>
+          <t>Post Basic Bachelor of Science [P.B.B.Sc] (Nursing)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Tuition Fee</t>
+          <t>Post Basic Bachelor of Science [P.B.B.Sc] (Nursing)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1,500</t>
+          <t>77,746</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2056,32 +2056,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>One-time Establishment Fee</t>
+          <t>Fellowship in Diabetology</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>One-time Establishment Fee</t>
+          <t>Fellowship in Diabetology</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>One-time Establishment Fee</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>1 L</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Full Time</t>
+          <t>Part Time</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -2118,27 +2118,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Other College Fees</t>
+          <t>MPT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Other College Fees</t>
+          <t>Master of Physiotherapy [MPT] (Orthopaedics)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Other College Fees</t>
+          <t>Master of Physiotherapy [MPT] (Orthopaedics)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>56,000</t>
+          <t>78,185</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2180,27 +2180,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Total College Fee</t>
+          <t>MOT</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Total College Fee</t>
+          <t>Master of Occupational Therapy [MOT] (Paediatrics)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Total College Fee</t>
+          <t>Master of Occupational Therapy [MOT] (Paediatrics)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.02 Lakhs</t>
+          <t>78,185</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2242,27 +2242,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>University Fee (incl. 18% GST)</t>
+          <t>Post Graduate Diploma in Hospital Administration</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>University Fee (incl. 18% GST)</t>
+          <t>Post Graduate Diploma in Hospital Administration</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>University Fee (incl. 18% GST)</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.73 Lakhs</t>
+          <t>48,793</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>NEET SS</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -2304,27 +2304,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Grand Total (All 3 Years)</t>
+          <t>PG Diploma Cardiac Technology</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Grand Total (All 3 Years)</t>
+          <t>PG Diploma Cardiac Technology</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Grand Total (All 3 Years)</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2.76 Lakhs</t>
+          <t>37,418</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2366,27 +2366,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>One-Time Establishment Fee</t>
+          <t>BPO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>One-Time Establishment Fee</t>
+          <t>Bachelor in Prosthetic and Orthotics [BPO]</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>One-Time Establishment Fee</t>
+          <t>Bachelor in Prosthetic and Orthotics [BPO]</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>1.7 L</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 years</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2428,27 +2428,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Other Charges</t>
+          <t>Ph.D</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Other Charges</t>
+          <t>Ph.D</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Other Charges</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>56,000</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>University Fee (Incl. GST)</t>
+          <t>Certificate Course in Laser Dentistry</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>University Fee (Incl. GST)</t>
+          <t>Certificate Course in Laser Dentistry</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>University Fee (Incl. GST)</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.73 Lakhs</t>
+          <t>62,000</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2552,27 +2552,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Total Fees</t>
+          <t>M.Tech</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Total Fees</t>
+          <t>Master of Technology [M.Tech] (Clinical Engineering)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Total Fees</t>
+          <t>Master of Technology [M.Tech] (Clinical Engineering)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2.76 Lakhs</t>
+          <t>28,660</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>GATE</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2614,27 +2614,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Indian Students</t>
+          <t>MOT</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Indian Students</t>
+          <t>Master in Occupational Therapy [MOT]</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Indian Students</t>
+          <t>Master in Occupational Therapy [MOT]</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.25 Lakhs (+ GST as per NBEMS)</t>
+          <t>78,185</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>11 Feb - 28 Mar 2026</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2676,27 +2676,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>International SAARC Nations</t>
+          <t>Fellowship</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>International SAARC Nations</t>
+          <t>Fellowship</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>International SAARC Nations</t>
+          <t>General</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.25 Lakhs (+ GST as per NBEMS)</t>
+          <t>29,340</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>GATE / UGC NET</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>
@@ -2738,27 +2738,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>International Non-SAARC Nations</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>International Non-SAARC Nations</t>
+          <t>Master of Surgery [MS] (Otorhinolaryngology)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>International Non-SAARC Nations</t>
+          <t>Master of Surgery [MS] (Otorhinolaryngology)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>USD 5,000</t>
+          <t>2.5 L</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2773,12 +2773,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>NEET PG</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>17 Apr - 07 Jul 2026</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2800,27 +2800,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hostel Security Deposit</t>
+          <t>DNB</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hostel Security Deposit</t>
+          <t>Diplomate National Board [DNB] (Palliative Medicine)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Hostel Security Deposit</t>
+          <t>Diplomate National Board [DNB] (Palliative Medicine)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>10,000 (refundable)</t>
+          <t>Not Specified</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>3 years</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2835,7 +2835,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>NEET PG</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>UG</t>
+          <t>PG</t>
         </is>
       </c>
     </row>
@@ -2862,27 +2862,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Approximate Monthly Living Expenses</t>
+          <t>B.Sc</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Approximate Monthly Living Expenses</t>
+          <t>Bachelor of Science [B.Sc] (Nursing)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Approximate Monthly Living Expenses</t>
+          <t>Bachelor of Science [B.Sc] (Nursing)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>8,000/month</t>
+          <t>1.6 Lakhs</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>10+2 with 45%</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2924,27 +2924,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Hostel Availability</t>
+          <t>BPT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Hostel Availability</t>
+          <t>Bachelor of Physiotherapy [BPT]</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Hostel Availability</t>
+          <t>Bachelor of Physiotherapy [BPT]</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Subject to availability at time of admission</t>
+          <t>1.36 Lakhs</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>4 Years</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Not Specified</t>
+          <t>10+2 with 35%</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2975,6 +2975,688 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Bachelor of Science [B.Sc]</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bachelor of Science [B.Sc]</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.4 Lakhs</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>4 Years</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>10+2 with 35%</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Doctor of Medicine [MD]</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Doctor of Medicine [MD]</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2.5 Lakhs</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>MBBS + NEET PG</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Tamil Nadu NEET PG Counselling, NEET PG</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>M.B.B.S.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>M.B.B.S.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2.9 Lakhs</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>5 Years</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>10+2 with 50% + NEET-UG</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>NEET, Tamil Nadu NEET Counselling</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>B.Sc. Nursing</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>B.Sc. Nursing</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.6 Lakhs</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>10+2 with 45%</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>BPT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>BPT</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>BPT</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.36 Lakhs</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>4 Years 6 Months</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>10+2 with 50%</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>B.Sc</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>B.Sc.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>B.Sc.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.35 – 1.42 lakh</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2.5 Lakh</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>MBBS + NEET PG</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>NEET PG</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>MBBS</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2.9 Lakh</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>5 Years 6 Months</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>10+2 with 50% + NEET-UG</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>NEET</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>UG</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>M.Ch</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2.76–3.07 Lakh</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Post-Graduation + NEET SS</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>NEET SS</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>M.Sc</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>68,185 – 1.03 Lakh</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2 Years</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>B.Sc. Nursing with 55%</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>IIT JAM</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>10343</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Fellowship</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Fellowship</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Fellowship</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>62,000</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>3-5 Years</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>MD/DNB</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>GATE / UGC NET</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Not Specified</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Doctorate</t>
         </is>
       </c>
     </row>

</xml_diff>